<commit_message>
Add SOH report for 2026-09-29
</commit_message>
<xml_diff>
--- a/reports/SOH_28_09_2026.xlsx
+++ b/reports/SOH_28_09_2026.xlsx
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>21000</v>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D20" s="2" t="n">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="E20" s="3" t="n">
         <v>0</v>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1268</v>
+        <v>1265</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>17000</v>
@@ -1861,7 +1861,7 @@
         </is>
       </c>
       <c r="D51" s="2" t="n">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="E51" s="3" t="n">
         <v>81000</v>
@@ -2197,7 +2197,7 @@
         </is>
       </c>
       <c r="D63" s="2" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="E63" s="3" t="n">
         <v>26500</v>
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>26500</v>
@@ -3793,7 +3793,7 @@
         </is>
       </c>
       <c r="D120" s="2" t="n">
-        <v>2534</v>
+        <v>2474</v>
       </c>
       <c r="E120" s="3" t="n">
         <v>3800</v>
@@ -4377,7 +4377,7 @@
         </is>
       </c>
       <c r="D141" s="2" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="E141" s="3" t="n">
         <v>11740</v>
@@ -4573,7 +4573,7 @@
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="E148" s="3" t="n">
         <v>34890</v>
@@ -6685,7 +6685,7 @@
         </is>
       </c>
       <c r="D226" s="2" t="n">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="E226" s="3" t="n">
         <v>1</v>
@@ -7609,7 +7609,7 @@
         </is>
       </c>
       <c r="D260" s="2" t="n">
-        <v>77</v>
+        <v>53</v>
       </c>
       <c r="E260" s="3" t="n">
         <v>24204</v>
@@ -8981,7 +8981,7 @@
         </is>
       </c>
       <c r="D309" s="2" t="n">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="E309" s="3" t="n">
         <v>26979</v>
@@ -9009,7 +9009,7 @@
         </is>
       </c>
       <c r="D310" s="2" t="n">
-        <v>505</v>
+        <v>493</v>
       </c>
       <c r="E310" s="3" t="n">
         <v>6682</v>
@@ -9121,7 +9121,7 @@
         </is>
       </c>
       <c r="D314" s="2" t="n">
-        <v>376</v>
+        <v>364</v>
       </c>
       <c r="E314" s="3" t="n">
         <v>17582</v>
@@ -9149,7 +9149,7 @@
         </is>
       </c>
       <c r="D315" s="2" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E315" s="3" t="n">
         <v>28228</v>
@@ -9177,7 +9177,7 @@
         </is>
       </c>
       <c r="D316" s="2" t="n">
-        <v>516</v>
+        <v>510</v>
       </c>
       <c r="E316" s="3" t="n">
         <v>39894</v>
@@ -9373,7 +9373,7 @@
         </is>
       </c>
       <c r="D323" s="2" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E323" s="3" t="n">
         <v>10962</v>
@@ -9429,7 +9429,7 @@
         </is>
       </c>
       <c r="D325" s="2" t="n">
-        <v>456</v>
+        <v>450</v>
       </c>
       <c r="E325" s="3" t="n">
         <v>12666</v>
@@ -12398,7 +12398,7 @@
         </is>
       </c>
       <c r="D431" s="2" t="n">
-        <v>145</v>
+        <v>121</v>
       </c>
       <c r="E431" s="3" t="n">
         <v>14565</v>
@@ -13098,7 +13098,7 @@
         </is>
       </c>
       <c r="D456" s="2" t="n">
-        <v>950</v>
+        <v>926</v>
       </c>
       <c r="E456" s="3" t="n">
         <v>9621</v>
@@ -13350,7 +13350,7 @@
         </is>
       </c>
       <c r="D465" s="2" t="n">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="E465" s="3" t="n">
         <v>11864</v>
@@ -13518,7 +13518,7 @@
         </is>
       </c>
       <c r="D471" s="2" t="n">
-        <v>731</v>
+        <v>707</v>
       </c>
       <c r="E471" s="3" t="n">
         <v>12104</v>
@@ -13742,7 +13742,7 @@
         </is>
       </c>
       <c r="D479" s="2" t="n">
-        <v>1845</v>
+        <v>1821</v>
       </c>
       <c r="E479" s="3" t="n">
         <v>15262</v>
@@ -14526,7 +14526,7 @@
         </is>
       </c>
       <c r="D507" s="2" t="n">
-        <v>282</v>
+        <v>258</v>
       </c>
       <c r="E507" s="3" t="n">
         <v>12504</v>
@@ -14554,7 +14554,7 @@
         </is>
       </c>
       <c r="D508" s="2" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E508" s="3" t="n">
         <v>7397</v>
@@ -16542,7 +16542,7 @@
         </is>
       </c>
       <c r="D579" s="2" t="n">
-        <v>173</v>
+        <v>137</v>
       </c>
       <c r="E579" s="3" t="n">
         <v>16732</v>
@@ -16654,7 +16654,7 @@
         </is>
       </c>
       <c r="D583" s="2" t="n">
-        <v>450</v>
+        <v>426</v>
       </c>
       <c r="E583" s="3" t="n">
         <v>9563</v>
@@ -16710,7 +16710,7 @@
         </is>
       </c>
       <c r="D585" s="2" t="n">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="E585" s="3" t="n">
         <v>17407</v>
@@ -20267,7 +20267,7 @@
         </is>
       </c>
       <c r="D712" s="2" t="n">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="E712" s="3" t="n">
         <v>8443</v>
@@ -23179,7 +23179,7 @@
         </is>
       </c>
       <c r="D816" s="2" t="n">
-        <v>462</v>
+        <v>450</v>
       </c>
       <c r="E816" s="3" t="n">
         <v>12738</v>
@@ -23207,7 +23207,7 @@
         </is>
       </c>
       <c r="D817" s="2" t="n">
-        <v>471</v>
+        <v>459</v>
       </c>
       <c r="E817" s="3" t="n">
         <v>16983</v>
@@ -23375,7 +23375,7 @@
         </is>
       </c>
       <c r="D823" s="2" t="n">
-        <v>169</v>
+        <v>145</v>
       </c>
       <c r="E823" s="3" t="n">
         <v>9239</v>
@@ -23488,7 +23488,7 @@
         </is>
       </c>
       <c r="D827" s="2" t="n">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="E827" s="3" t="n">
         <v>3900</v>
@@ -23712,7 +23712,7 @@
         </is>
       </c>
       <c r="D835" s="2" t="n">
-        <v>666</v>
+        <v>654</v>
       </c>
       <c r="E835" s="3" t="n">
         <v>17750</v>
@@ -23880,7 +23880,7 @@
         </is>
       </c>
       <c r="D841" s="2" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E841" s="3" t="n">
         <v>13122</v>
@@ -24272,7 +24272,7 @@
         </is>
       </c>
       <c r="D855" s="2" t="n">
-        <v>209</v>
+        <v>197</v>
       </c>
       <c r="E855" s="3" t="n">
         <v>14860</v>
@@ -24497,7 +24497,7 @@
         </is>
       </c>
       <c r="D863" s="2" t="n">
-        <v>1427</v>
+        <v>1415</v>
       </c>
       <c r="E863" s="3" t="n">
         <v>8181</v>
@@ -24637,7 +24637,7 @@
         </is>
       </c>
       <c r="D868" s="2" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E868" s="3" t="n">
         <v>9047</v>
@@ -24805,7 +24805,7 @@
         </is>
       </c>
       <c r="D874" s="2" t="n">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="E874" s="3" t="n">
         <v>8988</v>
@@ -28308,7 +28308,7 @@
         </is>
       </c>
       <c r="D999" s="2" t="n">
-        <v>370</v>
+        <v>358</v>
       </c>
       <c r="E999" s="3" t="n">
         <v>10871</v>
@@ -28644,7 +28644,7 @@
         </is>
       </c>
       <c r="D1011" s="2" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="E1011" s="3" t="n">
         <v>11795</v>
@@ -28868,7 +28868,7 @@
         </is>
       </c>
       <c r="D1019" s="2" t="n">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="E1019" s="3" t="n">
         <v>8060</v>
@@ -29288,7 +29288,7 @@
         </is>
       </c>
       <c r="D1034" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="E1034" s="3" t="n">
         <v>14684</v>
@@ -29513,7 +29513,7 @@
         </is>
       </c>
       <c r="D1042" s="2" t="n">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="E1042" s="3" t="n">
         <v>7008</v>
@@ -29681,7 +29681,7 @@
         </is>
       </c>
       <c r="D1048" s="2" t="n">
-        <v>269</v>
+        <v>245</v>
       </c>
       <c r="E1048" s="3" t="n">
         <v>6142</v>
@@ -30493,7 +30493,7 @@
         </is>
       </c>
       <c r="D1077" s="2" t="n">
-        <v>349</v>
+        <v>325</v>
       </c>
       <c r="E1077" s="3" t="n">
         <v>11027</v>
@@ -30773,7 +30773,7 @@
         </is>
       </c>
       <c r="D1087" s="2" t="n">
-        <v>1233</v>
+        <v>1221</v>
       </c>
       <c r="E1087" s="3" t="n">
         <v>5086</v>
@@ -30913,7 +30913,7 @@
         </is>
       </c>
       <c r="D1092" s="2" t="n">
-        <v>-6</v>
+        <v>0</v>
       </c>
       <c r="E1092" s="3" t="n">
         <v>13071</v>
@@ -31025,7 +31025,7 @@
         </is>
       </c>
       <c r="D1096" s="2" t="n">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="E1096" s="3" t="n">
         <v>40981</v>
@@ -32397,7 +32397,7 @@
         </is>
       </c>
       <c r="D1145" s="2" t="n">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="E1145" s="3" t="n">
         <v>14752</v>
@@ -32537,7 +32537,7 @@
         </is>
       </c>
       <c r="D1150" s="2" t="n">
-        <v>466</v>
+        <v>460</v>
       </c>
       <c r="E1150" s="3" t="n">
         <v>8325</v>
@@ -32593,7 +32593,7 @@
         </is>
       </c>
       <c r="D1152" s="2" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="E1152" s="3" t="n">
         <v>8155</v>
@@ -32789,7 +32789,7 @@
         </is>
       </c>
       <c r="D1159" s="2" t="n">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="E1159" s="3" t="n">
         <v>3391</v>
@@ -35701,7 +35701,7 @@
         </is>
       </c>
       <c r="D1263" s="2" t="n">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E1263" s="3" t="n">
         <v>13998</v>
@@ -35953,7 +35953,7 @@
         </is>
       </c>
       <c r="D1272" s="2" t="n">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="E1272" s="3" t="n">
         <v>10600</v>
@@ -36009,7 +36009,7 @@
         </is>
       </c>
       <c r="D1274" s="2" t="n">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E1274" s="3" t="n">
         <v>22663</v>
@@ -36149,7 +36149,7 @@
         </is>
       </c>
       <c r="D1279" s="2" t="n">
-        <v>509</v>
+        <v>497</v>
       </c>
       <c r="E1279" s="3" t="n">
         <v>25495</v>
@@ -36205,7 +36205,7 @@
         </is>
       </c>
       <c r="D1281" s="2" t="n">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="E1281" s="3" t="n">
         <v>13595</v>
@@ -36877,7 +36877,7 @@
         </is>
       </c>
       <c r="D1305" s="2" t="n">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E1305" s="3" t="n">
         <v>8429</v>
@@ -36961,7 +36961,7 @@
         </is>
       </c>
       <c r="D1308" s="2" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E1308" s="3" t="n">
         <v>14160</v>
@@ -37549,7 +37549,7 @@
         </is>
       </c>
       <c r="D1329" s="2" t="n">
-        <v>923</v>
+        <v>899</v>
       </c>
       <c r="E1329" s="3" t="n">
         <v>7174</v>
@@ -39705,7 +39705,7 @@
         </is>
       </c>
       <c r="D1406" s="2" t="n">
-        <v>2041</v>
+        <v>1993</v>
       </c>
       <c r="E1406" s="3" t="n">
         <v>11094</v>
@@ -39733,7 +39733,7 @@
         </is>
       </c>
       <c r="D1407" s="2" t="n">
-        <v>1847</v>
+        <v>1823</v>
       </c>
       <c r="E1407" s="3" t="n">
         <v>10548</v>
@@ -40657,7 +40657,7 @@
         </is>
       </c>
       <c r="D1440" s="2" t="n">
-        <v>144</v>
+        <v>96</v>
       </c>
       <c r="E1440" s="3" t="n">
         <v>10733</v>
@@ -41665,7 +41665,7 @@
         </is>
       </c>
       <c r="D1476" s="2" t="n">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="E1476" s="3" t="n">
         <v>16495</v>
@@ -41861,7 +41861,7 @@
         </is>
       </c>
       <c r="D1483" s="2" t="n">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="E1483" s="3" t="n">
         <v>6659</v>
@@ -41973,7 +41973,7 @@
         </is>
       </c>
       <c r="D1487" s="2" t="n">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="E1487" s="3" t="n">
         <v>6659</v>
@@ -42589,7 +42589,7 @@
         </is>
       </c>
       <c r="D1509" s="2" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E1509" s="3" t="n">
         <v>41300</v>
@@ -43935,7 +43935,7 @@
         </is>
       </c>
       <c r="D1557" s="2" t="n">
-        <v>546</v>
+        <v>534</v>
       </c>
       <c r="E1557" s="3" t="n">
         <v>19684</v>

</xml_diff>